<commit_message>
add week report template
</commit_message>
<xml_diff>
--- a/planning/Project_Tracker_HK1_Nguyen_Hai_Minh.xlsx
+++ b/planning/Project_Tracker_HK1_Nguyen_Hai_Minh.xlsx
@@ -6,17 +6,19 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Plan" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Chi tiet HK1" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bao cao tuan" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hoc RV32I tuan" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Bao cao tuan'!$1:$6</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="2">'Bao cao tuan'!$A$1:$L$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Hoc RV32I tuan'!$A$3:$L$10</definedName>
   </definedNames>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="9">
     <numFmt numFmtId="164" formatCode="mmm\ d"/>
     <numFmt numFmtId="165" formatCode="#,##0;[Red]\(#,##0\);\-"/>
     <numFmt numFmtId="166" formatCode=";;;"/>
@@ -25,8 +27,9 @@
     <numFmt numFmtId="169" formatCode="dd/mm/yy"/>
     <numFmt numFmtId="170" formatCode="dd/mm"/>
     <numFmt numFmtId="171" formatCode="0.0"/>
+    <numFmt numFmtId="172" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="29">
     <font>
       <name val="Arial"/>
       <sz val="11"/>
@@ -196,6 +199,12 @@
       <color rgb="000563C1"/>
       <sz val="11"/>
       <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="17">
@@ -578,7 +587,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="155">
+  <cellXfs count="156">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1014,6 +1023,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1458,7 +1470,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AD68"/>
+  <dimension ref="A1:AD68"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="3.33203125" customWidth="1" style="14" min="1" max="1"/>
@@ -1474,6 +1486,7 @@
     <col width="8.83203125" customWidth="1" style="14" min="31" max="16384"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="32" customHeight="1">
       <c r="B2" s="19" t="inlineStr">
         <is>
@@ -5521,6 +5534,8 @@
       <c r="AC42" s="136" t="n"/>
       <c r="AD42" s="137" t="n"/>
     </row>
+    <row r="43"/>
+    <row r="44"/>
     <row r="45" ht="24" customHeight="1">
       <c r="B45" s="94" t="inlineStr">
         <is>
@@ -6576,7 +6591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:N60"/>
+  <dimension ref="A1:N60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3.299999952316284" customWidth="1" min="1" max="1"/>
@@ -6595,6 +6610,7 @@
     <col width="12" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="32" customHeight="1">
       <c r="B2" s="60" t="inlineStr">
         <is>
@@ -6745,7 +6761,7 @@
       <c r="J8" s="70" t="str"/>
       <c r="K8" s="70" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R8 (sách chính); R1</t>
         </is>
       </c>
       <c r="L8" s="144">
@@ -6797,7 +6813,7 @@
       </c>
       <c r="K9" s="73" t="inlineStr">
         <is>
-          <t>R1; R3 bổ trợ</t>
+          <t>R8 (sách chính); R1; R3 bổ trợ</t>
         </is>
       </c>
       <c r="L9" s="147">
@@ -6849,7 +6865,7 @@
       </c>
       <c r="K10" s="70" t="inlineStr">
         <is>
-          <t>R1; R2; R4 tra cứu</t>
+          <t>R8 (sách chính); R1; R2; R4 tra cứu</t>
         </is>
       </c>
       <c r="L10" s="144">
@@ -6901,7 +6917,7 @@
       </c>
       <c r="K11" s="73" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R8 (sách chính); R1</t>
         </is>
       </c>
       <c r="L11" s="147">
@@ -6953,7 +6969,7 @@
       </c>
       <c r="K12" s="70" t="inlineStr">
         <is>
-          <t>R1; R2</t>
+          <t>R8 (sách chính); R1; R2</t>
         </is>
       </c>
       <c r="L12" s="144">
@@ -7005,7 +7021,7 @@
       </c>
       <c r="K13" s="73" t="inlineStr">
         <is>
-          <t>R1; R2</t>
+          <t>R8 (sách chính); R1; R2</t>
         </is>
       </c>
       <c r="L13" s="147">
@@ -7057,7 +7073,7 @@
       </c>
       <c r="K14" s="70" t="inlineStr">
         <is>
-          <t>R1; R5 hoặc R6</t>
+          <t>R8 (sách chính); R1; R5 hoặc R6</t>
         </is>
       </c>
       <c r="L14" s="144">
@@ -7161,7 +7177,7 @@
       </c>
       <c r="K16" s="70" t="inlineStr">
         <is>
-          <t>R1; tài liệu tool của board</t>
+          <t>R8 (sách chính); R1; tài liệu tool của board</t>
         </is>
       </c>
       <c r="L16" s="144">
@@ -7213,7 +7229,7 @@
       </c>
       <c r="K17" s="73" t="inlineStr">
         <is>
-          <t>R4; R5 hoặc R6</t>
+          <t>R8 (sách chính); R4; R5 hoặc R6</t>
         </is>
       </c>
       <c r="L17" s="147">
@@ -8500,7 +8516,7 @@
       </c>
       <c r="H50" s="70" t="inlineStr">
         <is>
-          <t>Sách chính theo lựa chọn ngày 24/10/2026; dùng cho các buổi học kiến trúc tiếp theo. Đối chiếu chương/mục trong PDF trước mỗi phần đọc; chưa ghi nhận đã đọc.</t>
+          <t>Sách chính: §1.3; §1.9 tr.52–53; A.9; C.1. Đã đối chiếu các đoạn liên quan để soạn bài ngày 26/10; chưa xác nhận tiến độ học viên. Bài tập RV32I đối chiếu R4.</t>
         </is>
       </c>
       <c r="K50" s="70" t="inlineStr">
@@ -8527,7 +8543,7 @@
     <row r="52" ht="25" customHeight="1">
       <c r="B52" s="62" t="inlineStr">
         <is>
-          <t>Tuần 1 làm C01 + P01: tự đánh giá kỹ năng, biểu diễn số/con trỏ, chạy tổng mảng, ghi scope và nguồn lực. Cuối tuần cập nhật trạng thái, giờ thực tế, bằng chứng và câu hỏi còn vướng. Sao chép URL trong danh mục để mở học liệu.</t>
+          <t>Ưu tiên 26/10–01/11: tab Hoc RV32I tuan, 10 giờ dự kiến học và dựng các khối T3 cho BTL. Đây là phân bổ tuần đang làm, không cộng thêm tải Gantt cũ. Trạng thái Cxx/Pxx chỉ đổi khi có bằng chứng thực tế.</t>
         </is>
       </c>
     </row>
@@ -8616,6 +8632,7 @@
     <mergeCell ref="B55:N57"/>
     <mergeCell ref="C47:G47"/>
     <mergeCell ref="K49:N49"/>
+    <mergeCell ref="C50:G50"/>
     <mergeCell ref="C44:G44"/>
     <mergeCell ref="H47:J47"/>
     <mergeCell ref="H48:J48"/>
@@ -8627,14 +8644,13 @@
     <mergeCell ref="B2:N2"/>
     <mergeCell ref="C48:G48"/>
     <mergeCell ref="H43:J43"/>
+    <mergeCell ref="K50:N50"/>
     <mergeCell ref="K44:N44"/>
     <mergeCell ref="K46:N46"/>
+    <mergeCell ref="H50:J50"/>
     <mergeCell ref="H44:J44"/>
     <mergeCell ref="B4:N5"/>
     <mergeCell ref="K43:N43"/>
-    <mergeCell ref="C50:G50"/>
-    <mergeCell ref="H50:J50"/>
-    <mergeCell ref="K50:N50"/>
   </mergeCells>
   <conditionalFormatting sqref="E8:F37">
     <cfRule type="expression" priority="1" dxfId="11">
@@ -8661,7 +8677,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:M26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -8676,6 +8692,7 @@
     <col width="19" customWidth="1" min="10" max="10"/>
     <col width="40" customWidth="1" min="11" max="11"/>
     <col width="42" customWidth="1" min="12" max="12"/>
+    <col width="55" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="31" customHeight="1">
@@ -8688,10 +8705,11 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="149" t="inlineStr">
         <is>
-          <t>Ghi ngắn: tiến độ tuần này → khó khăn và cách giải quyết → nhiệm vụ tuần tới. Báo cáo Word dùng để gửi thầy; ghi ngày gửi/góp ý sau khi thực hiện.</t>
-        </is>
-      </c>
-    </row>
+          <t>Mỗi tuần thứ Hai–Chủ nhật: tiến độ → vấn đề → giải pháp → ý nghĩa thiết kế → kế hoạch tới. Chỉ ghi ngày gửi sau khi thực hiện.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="149" t="inlineStr">
         <is>
@@ -8699,7 +8717,7 @@
         </is>
       </c>
       <c r="B4" s="150" t="n">
-        <v>46316</v>
+        <v>46321</v>
       </c>
       <c r="D4" s="149" t="inlineStr">
         <is>
@@ -8707,6 +8725,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6" ht="32" customHeight="1">
       <c r="A6" s="151" t="inlineStr">
         <is>
@@ -8766,6 +8785,11 @@
       <c r="L6" s="151" t="inlineStr">
         <is>
           <t>Việc cần làm sau góp ý</t>
+        </is>
+      </c>
+      <c r="M6" s="151" t="inlineStr">
+        <is>
+          <t>Ý nghĩa thiết kế</t>
         </is>
       </c>
     </row>
@@ -8783,37 +8807,42 @@
       </c>
       <c r="D7" s="152" t="inlineStr">
         <is>
-          <t>Đã có khung workspace, đề cương và tracker; học viên đã gom source vào Project_source/. Bản báo cáo tuần 01 đang là nháp.</t>
+          <t>Đã tổ chức sách/bài báo, soạn bài học Word và lịch thực hành; đọc cấu trúc T3. Chưa xác nhận học viên hoàn thành khối hoặc mô phỏng.</t>
         </is>
       </c>
       <c r="E7" s="152" t="inlineStr">
         <is>
-          <t>Board chưa chốt; môi trường triển khai chưa ghi nhận đầy đủ.</t>
+          <t>Cần nối ví dụ RV64G trong sách với RV32I; T3 còn control tay; cần kiểm chứng U-immediate.</t>
         </is>
       </c>
       <c r="F7" s="152" t="inlineStr">
         <is>
-          <t>Khảo sát board có thể tiếp cận; học viên tự chuẩn bị môi trường, bổ sung kết quả thực tế.</t>
+          <t>Bài học có nguồn/mục/trang, ví dụ giải và vector expected; kiểm chứng từng khối trong Logisim, ghi actual khi thực hành.</t>
         </is>
       </c>
       <c r="G7" s="152" t="inlineStr">
         <is>
-          <t>Đọc kiến trúc Ibex/core-SoC; khảo sát board; chuẩn bị môi trường theo điều kiện thực tế.</t>
+          <t>02–08/11: hoàn tất khối tồn đọng; control, memory và chương trình ROM tự chạy; chỉ học pipeline sau single-cycle ổn định.</t>
         </is>
       </c>
       <c r="H7" s="154" t="inlineStr">
         <is>
-          <t>weekly/Bao_cao_tuan_01_2026-10-21_2026-10-27.docx</t>
+          <t>weekly/Bao_cao_tuan_01_2026-10-26_2026-11-01.docx</t>
         </is>
       </c>
       <c r="I7" s="153" t="n"/>
       <c r="J7" s="152" t="inlineStr">
         <is>
-          <t>Đang soạn</t>
+          <t>Đang soạn; chưa gửi</t>
         </is>
       </c>
       <c r="K7" s="152" t="n"/>
       <c r="L7" s="152" t="n"/>
+      <c r="M7" s="152" t="inlineStr">
+        <is>
+          <t>Mục tiêu: state/clock, 2R1W, ALUSrc, branch target/decision; học viên bổ sung kết luận sau thực hành.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="46" customHeight="1">
       <c r="A8" s="152" t="n">
@@ -8840,6 +8869,7 @@
       </c>
       <c r="K8" s="152" t="n"/>
       <c r="L8" s="152" t="n"/>
+      <c r="M8" s="152" t="n"/>
     </row>
     <row r="9" ht="46" customHeight="1">
       <c r="A9" s="152" t="n">
@@ -8866,6 +8896,7 @@
       </c>
       <c r="K9" s="152" t="n"/>
       <c r="L9" s="152" t="n"/>
+      <c r="M9" s="152" t="n"/>
     </row>
     <row r="10" ht="46" customHeight="1">
       <c r="A10" s="152" t="n">
@@ -8892,6 +8923,7 @@
       </c>
       <c r="K10" s="152" t="n"/>
       <c r="L10" s="152" t="n"/>
+      <c r="M10" s="152" t="n"/>
     </row>
     <row r="11" ht="46" customHeight="1">
       <c r="A11" s="152" t="n">
@@ -8918,6 +8950,7 @@
       </c>
       <c r="K11" s="152" t="n"/>
       <c r="L11" s="152" t="n"/>
+      <c r="M11" s="152" t="n"/>
     </row>
     <row r="12" ht="46" customHeight="1">
       <c r="A12" s="152" t="n">
@@ -8944,6 +8977,7 @@
       </c>
       <c r="K12" s="152" t="n"/>
       <c r="L12" s="152" t="n"/>
+      <c r="M12" s="152" t="n"/>
     </row>
     <row r="13" ht="46" customHeight="1">
       <c r="A13" s="152" t="n">
@@ -8970,6 +9004,7 @@
       </c>
       <c r="K13" s="152" t="n"/>
       <c r="L13" s="152" t="n"/>
+      <c r="M13" s="152" t="n"/>
     </row>
     <row r="14" ht="46" customHeight="1">
       <c r="A14" s="152" t="n">
@@ -8996,6 +9031,7 @@
       </c>
       <c r="K14" s="152" t="n"/>
       <c r="L14" s="152" t="n"/>
+      <c r="M14" s="152" t="n"/>
     </row>
     <row r="15" ht="46" customHeight="1">
       <c r="A15" s="152" t="n">
@@ -9022,6 +9058,7 @@
       </c>
       <c r="K15" s="152" t="n"/>
       <c r="L15" s="152" t="n"/>
+      <c r="M15" s="152" t="n"/>
     </row>
     <row r="16" ht="46" customHeight="1">
       <c r="A16" s="152" t="n">
@@ -9048,6 +9085,7 @@
       </c>
       <c r="K16" s="152" t="n"/>
       <c r="L16" s="152" t="n"/>
+      <c r="M16" s="152" t="n"/>
     </row>
     <row r="17" ht="46" customHeight="1">
       <c r="A17" s="152" t="n">
@@ -9074,6 +9112,7 @@
       </c>
       <c r="K17" s="152" t="n"/>
       <c r="L17" s="152" t="n"/>
+      <c r="M17" s="152" t="n"/>
     </row>
     <row r="18" ht="46" customHeight="1">
       <c r="A18" s="152" t="n">
@@ -9100,6 +9139,7 @@
       </c>
       <c r="K18" s="152" t="n"/>
       <c r="L18" s="152" t="n"/>
+      <c r="M18" s="152" t="n"/>
     </row>
     <row r="19" ht="46" customHeight="1">
       <c r="A19" s="152" t="n">
@@ -9126,6 +9166,7 @@
       </c>
       <c r="K19" s="152" t="n"/>
       <c r="L19" s="152" t="n"/>
+      <c r="M19" s="152" t="n"/>
     </row>
     <row r="20" ht="46" customHeight="1">
       <c r="A20" s="152" t="n">
@@ -9152,6 +9193,7 @@
       </c>
       <c r="K20" s="152" t="n"/>
       <c r="L20" s="152" t="n"/>
+      <c r="M20" s="152" t="n"/>
     </row>
     <row r="21" ht="46" customHeight="1">
       <c r="A21" s="152" t="n">
@@ -9178,6 +9220,7 @@
       </c>
       <c r="K21" s="152" t="n"/>
       <c r="L21" s="152" t="n"/>
+      <c r="M21" s="152" t="n"/>
     </row>
     <row r="22" ht="46" customHeight="1">
       <c r="A22" s="152" t="n">
@@ -9204,6 +9247,7 @@
       </c>
       <c r="K22" s="152" t="n"/>
       <c r="L22" s="152" t="n"/>
+      <c r="M22" s="152" t="n"/>
     </row>
     <row r="23" ht="46" customHeight="1">
       <c r="A23" s="152" t="n">
@@ -9230,6 +9274,7 @@
       </c>
       <c r="K23" s="152" t="n"/>
       <c r="L23" s="152" t="n"/>
+      <c r="M23" s="152" t="n"/>
     </row>
     <row r="24" ht="46" customHeight="1">
       <c r="A24" s="152" t="n">
@@ -9256,6 +9301,7 @@
       </c>
       <c r="K24" s="152" t="n"/>
       <c r="L24" s="152" t="n"/>
+      <c r="M24" s="152" t="n"/>
     </row>
     <row r="25" ht="46" customHeight="1">
       <c r="A25" s="152" t="n">
@@ -9282,6 +9328,7 @@
       </c>
       <c r="K25" s="152" t="n"/>
       <c r="L25" s="152" t="n"/>
+      <c r="M25" s="152" t="n"/>
     </row>
     <row r="26" ht="46" customHeight="1">
       <c r="A26" s="152" t="n">
@@ -9308,6 +9355,7 @@
       </c>
       <c r="K26" s="152" t="n"/>
       <c r="L26" s="152" t="n"/>
+      <c r="M26" s="152" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -9330,4 +9378,460 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:L11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="39" customWidth="1" min="3" max="3"/>
+    <col width="49" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="155" t="inlineStr">
+        <is>
+          <t>KẾ HOẠCH HỌC RV32I • 26/10–01/11/2026</t>
+        </is>
+      </c>
+      <c r="B1" s="155" t="n"/>
+      <c r="C1" s="155" t="n"/>
+      <c r="D1" s="155" t="n"/>
+      <c r="E1" s="155" t="n"/>
+      <c r="F1" s="155" t="n"/>
+      <c r="G1" s="155" t="n"/>
+      <c r="H1" s="155" t="n"/>
+      <c r="I1" s="155" t="n"/>
+      <c r="J1" s="155" t="n"/>
+      <c r="K1" s="155" t="n"/>
+      <c r="L1" s="155" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="155" t="inlineStr">
+        <is>
+          <t>10 giờ dự kiến; ưu tiên tuần này thay phân bổ chi tiết cũ. Không đánh dấu hoàn thành mã học kỳ từ việc soạn tài liệu.</t>
+        </is>
+      </c>
+      <c r="B2" s="155" t="n"/>
+      <c r="C2" s="155" t="n"/>
+      <c r="D2" s="155" t="n"/>
+      <c r="E2" s="155" t="n"/>
+      <c r="F2" s="155" t="n"/>
+      <c r="G2" s="155" t="n"/>
+      <c r="H2" s="155" t="n"/>
+      <c r="I2" s="155" t="n"/>
+      <c r="J2" s="155" t="n"/>
+      <c r="K2" s="155" t="n"/>
+      <c r="L2" s="155" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="155" t="inlineStr">
+        <is>
+          <t>Ngày</t>
+        </is>
+      </c>
+      <c r="B3" s="155" t="inlineStr">
+        <is>
+          <t>Giờ dự kiến</t>
+        </is>
+      </c>
+      <c r="C3" s="155" t="inlineStr">
+        <is>
+          <t>Nội dung</t>
+        </is>
+      </c>
+      <c r="D3" s="155" t="inlineStr">
+        <is>
+          <t>Đầu ra / điều kiện hoàn thành</t>
+        </is>
+      </c>
+      <c r="E3" s="155" t="inlineStr">
+        <is>
+          <t>Mã liên hệ</t>
+        </is>
+      </c>
+      <c r="F3" s="155" t="inlineStr">
+        <is>
+          <t>Nguồn</t>
+        </is>
+      </c>
+      <c r="G3" s="155" t="inlineStr">
+        <is>
+          <t>Trạng thái học</t>
+        </is>
+      </c>
+      <c r="H3" s="155" t="inlineStr">
+        <is>
+          <t>Giờ thực tế</t>
+        </is>
+      </c>
+      <c r="I3" s="155" t="inlineStr">
+        <is>
+          <t>Bằng chứng</t>
+        </is>
+      </c>
+      <c r="J3" s="155" t="inlineStr">
+        <is>
+          <t>Vấn đề / giải pháp</t>
+        </is>
+      </c>
+      <c r="K3" s="155" t="inlineStr">
+        <is>
+          <t>Ý nghĩa thiết kế</t>
+        </is>
+      </c>
+      <c r="L3" s="155" t="inlineStr">
+        <is>
+          <t>Bài học Word</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="75" customHeight="1">
+      <c r="A4" s="153" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B4" s="152" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C4" s="152" t="inlineStr">
+        <is>
+          <t>Buổi 1: trạng thái, clock, PC</t>
+        </is>
+      </c>
+      <c r="D4" s="152" t="inlineStr">
+        <is>
+          <t>Sơ đồ PC + bảng trước/sau cạnh</t>
+        </is>
+      </c>
+      <c r="E4" s="152" t="inlineStr">
+        <is>
+          <t>C01/C02</t>
+        </is>
+      </c>
+      <c r="F4" s="152" t="inlineStr">
+        <is>
+          <t>S1, S3, S4</t>
+        </is>
+      </c>
+      <c r="G4" s="152" t="inlineStr">
+        <is>
+          <t>Chưa thực hiện</t>
+        </is>
+      </c>
+      <c r="H4" s="152" t="n"/>
+      <c r="I4" s="152" t="n"/>
+      <c r="J4" s="152" t="n"/>
+      <c r="K4" s="152" t="n"/>
+      <c r="L4" s="152" t="inlineStr">
+        <is>
+          <t>Bài học Word</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="75" customHeight="1">
+      <c r="A5" s="153" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B5" s="152" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C5" s="152" t="inlineStr">
+        <is>
+          <t>Buổi 2: fetch và decode</t>
+        </is>
+      </c>
+      <c r="D5" s="152" t="inlineStr">
+        <is>
+          <t>Hai lệnh đã tách field + ROM index</t>
+        </is>
+      </c>
+      <c r="E5" s="152" t="inlineStr">
+        <is>
+          <t>C03</t>
+        </is>
+      </c>
+      <c r="F5" s="152" t="inlineStr">
+        <is>
+          <t>S3, S4, T3</t>
+        </is>
+      </c>
+      <c r="G5" s="152" t="inlineStr">
+        <is>
+          <t>Chưa thực hiện</t>
+        </is>
+      </c>
+      <c r="H5" s="152" t="n"/>
+      <c r="I5" s="152" t="n"/>
+      <c r="J5" s="152" t="n"/>
+      <c r="K5" s="152" t="n"/>
+      <c r="L5" s="152" t="inlineStr">
+        <is>
+          <t>Bài học Word</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="75" customHeight="1">
+      <c r="A6" s="153" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B6" s="152" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="152" t="inlineStr">
+        <is>
+          <t>Buổi 3: register file và ALU</t>
+        </is>
+      </c>
+      <c r="D6" s="152" t="inlineStr">
+        <is>
+          <t>Kiểm tra cổng ghi/x0 + 11 vector ALU</t>
+        </is>
+      </c>
+      <c r="E6" s="152" t="inlineStr">
+        <is>
+          <t>C02/C03</t>
+        </is>
+      </c>
+      <c r="F6" s="152" t="inlineStr">
+        <is>
+          <t>S3, T3</t>
+        </is>
+      </c>
+      <c r="G6" s="152" t="inlineStr">
+        <is>
+          <t>Chưa thực hiện</t>
+        </is>
+      </c>
+      <c r="H6" s="152" t="n"/>
+      <c r="I6" s="152" t="n"/>
+      <c r="J6" s="152" t="n"/>
+      <c r="K6" s="152" t="n"/>
+      <c r="L6" s="152" t="inlineStr">
+        <is>
+          <t>Bài học Word</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="75" customHeight="1">
+      <c r="A7" s="153" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B7" s="152" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C7" s="152" t="inlineStr">
+        <is>
+          <t>Buổi 4: immediate và ALUSrc</t>
+        </is>
+      </c>
+      <c r="D7" s="152" t="inlineStr">
+        <is>
+          <t>6 vector immediate + ADDI âm</t>
+        </is>
+      </c>
+      <c r="E7" s="152" t="inlineStr">
+        <is>
+          <t>C03/C05</t>
+        </is>
+      </c>
+      <c r="F7" s="152" t="inlineStr">
+        <is>
+          <t>S3, ISA, T3</t>
+        </is>
+      </c>
+      <c r="G7" s="152" t="inlineStr">
+        <is>
+          <t>Chưa thực hiện</t>
+        </is>
+      </c>
+      <c r="H7" s="152" t="n"/>
+      <c r="I7" s="152" t="n"/>
+      <c r="J7" s="152" t="n"/>
+      <c r="K7" s="152" t="n"/>
+      <c r="L7" s="152" t="inlineStr">
+        <is>
+          <t>Bài học Word</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="75" customHeight="1">
+      <c r="A8" s="153" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B8" s="152" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C8" s="152" t="inlineStr">
+        <is>
+          <t>Buổi 5: ghép datapath và PC</t>
+        </is>
+      </c>
+      <c r="D8" s="152" t="inlineStr">
+        <is>
+          <t>Trace ADD/ADDI + 3 tình huống PC</t>
+        </is>
+      </c>
+      <c r="E8" s="152" t="inlineStr">
+        <is>
+          <t>C05</t>
+        </is>
+      </c>
+      <c r="F8" s="152" t="inlineStr">
+        <is>
+          <t>S3, S4, ISA, T3</t>
+        </is>
+      </c>
+      <c r="G8" s="152" t="inlineStr">
+        <is>
+          <t>Chưa thực hiện</t>
+        </is>
+      </c>
+      <c r="H8" s="152" t="n"/>
+      <c r="I8" s="152" t="n"/>
+      <c r="J8" s="152" t="n"/>
+      <c r="K8" s="152" t="n"/>
+      <c r="L8" s="152" t="inlineStr">
+        <is>
+          <t>Bài học Word</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="75" customHeight="1">
+      <c r="A9" s="153" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B9" s="152" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="152" t="inlineStr">
+        <is>
+          <t>Buổi 6: ý nghĩa và hiệu năng</t>
+        </is>
+      </c>
+      <c r="D9" s="152" t="inlineStr">
+        <is>
+          <t>Bài tính time + giải thích liên hệ Ibex</t>
+        </is>
+      </c>
+      <c r="E9" s="152" t="inlineStr">
+        <is>
+          <t>C05/C09</t>
+        </is>
+      </c>
+      <c r="F9" s="152" t="inlineStr">
+        <is>
+          <t>S1, S2, S4</t>
+        </is>
+      </c>
+      <c r="G9" s="152" t="inlineStr">
+        <is>
+          <t>Chưa thực hiện</t>
+        </is>
+      </c>
+      <c r="H9" s="152" t="n"/>
+      <c r="I9" s="152" t="n"/>
+      <c r="J9" s="152" t="n"/>
+      <c r="K9" s="152" t="n"/>
+      <c r="L9" s="152" t="inlineStr">
+        <is>
+          <t>Bài học Word</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="75" customHeight="1">
+      <c r="A10" s="153" t="n">
+        <v>46327</v>
+      </c>
+      <c r="B10" s="152" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="152" t="inlineStr">
+        <is>
+          <t>Rà soát và viết báo cáo tuần</t>
+        </is>
+      </c>
+      <c r="D10" s="152" t="inlineStr">
+        <is>
+          <t>Kết quả thật, vấn đề, giải pháp, ý nghĩa, kế hoạch tới</t>
+        </is>
+      </c>
+      <c r="E10" s="152" t="inlineStr">
+        <is>
+          <t>Báo cáo GVHD</t>
+        </is>
+      </c>
+      <c r="F10" s="152" t="inlineStr">
+        <is>
+          <t>Báo cáo tuần 01</t>
+        </is>
+      </c>
+      <c r="G10" s="152" t="inlineStr">
+        <is>
+          <t>Chưa thực hiện</t>
+        </is>
+      </c>
+      <c r="H10" s="152" t="n"/>
+      <c r="I10" s="152" t="n"/>
+      <c r="J10" s="152" t="n"/>
+      <c r="K10" s="152" t="n"/>
+      <c r="L10" s="152" t="inlineStr">
+        <is>
+          <t>Bài học Word</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="152" t="inlineStr">
+        <is>
+          <t>Tổng</t>
+        </is>
+      </c>
+      <c r="B11" s="152">
+        <f>SUM(B4:B10)</f>
+        <v/>
+      </c>
+      <c r="C11" s="152" t="n"/>
+      <c r="D11" s="152" t="n"/>
+      <c r="E11" s="152" t="n"/>
+      <c r="F11" s="152" t="n"/>
+      <c r="G11" s="152" t="n"/>
+      <c r="H11" s="152" t="n"/>
+      <c r="I11" s="152" t="n"/>
+      <c r="J11" s="152" t="n"/>
+      <c r="K11" s="152" t="n"/>
+      <c r="L11" s="152" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:L10"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A1:L1"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L4" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L5" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L6" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L7" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L10" r:id="rId7"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="1" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>